<commit_message>
Refresh spreadsheet — Fever CV built
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job Candidates.xlsx
+++ b/Job Candidates.xlsx
@@ -666,7 +666,7 @@
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>Generalist PM. Archetype A. Confirms the JD Joaco already has a skill-gap-map for (CV and JDs/jds/n26-oae.md) is still live as of 2026-08-11. CV in Opportunities/N26 - Ops Automation Enablement/.</t>
+          <t>Generalist PM. Archetype A. Confirms the JD Joaco already has a skill-gap-map for (CV and JDs/jds/n26-oae.md) is still live as of 2026-08-11. CV in Opportunities/26-08-25 - N26 - Ops Automation Enablement/.</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>Generalist PM. Archetype B, direct KYC domain match (same angle as the IOL story). Barcelona. CV in Opportunities/Spendesk - KYC AML/.</t>
+          <t>Generalist PM. Archetype B, direct KYC domain match (same angle as the IOL story). Barcelona. CV in Opportunities/26-08-25 - Spendesk - KYC AML/.</t>
         </is>
       </c>
     </row>
@@ -782,7 +782,7 @@
       </c>
       <c r="L4" s="5" t="inlineStr">
         <is>
-          <t>Technical Specialist PM, Medium proximity (best-odds one of today's technical-specialist leads). Archetype B, payments. Barcelona. Real gap: JD marks national payment-scheme participation (SEPA/FPS/ACH) as mandatory; Xepelin's bank integrations are a real bridge, not scheme-level but closer than any other technical lead today. See Opportunities/Thunes - Global Accounts/tailoring-notes.md.</t>
+          <t>Technical Specialist PM, Medium proximity (best-odds one of today's technical-specialist leads). Archetype B, payments. Barcelona. Real gap: JD marks national payment-scheme participation (SEPA/FPS/ACH) as mandatory; Xepelin's bank integrations are a real bridge, not scheme-level but closer than any other technical lead today. See Opportunities/26-08-25 - Thunes - Global Accounts/tailoring-notes.md.</t>
         </is>
       </c>
     </row>
@@ -840,7 +840,7 @@
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>Generalist PM. Archetype A — FP&amp;A software, not fintech-core but ops-automation core. Barcelona. JD explicitly welcomes ambiguous cross-functional backgrounds. CV in Opportunities/Abacum - AI Adoption Enablement/.</t>
+          <t>Generalist PM. Archetype A — FP&amp;A software, not fintech-core but ops-automation core. Barcelona. JD explicitly welcomes ambiguous cross-functional backgrounds. CV in Opportunities/26-08-25 - Abacum - AI Adoption Enablement/.</t>
         </is>
       </c>
     </row>
@@ -902,7 +902,7 @@
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>Generalist PM. Archetype C — AI-native product startup, explicitly domain-agnostic. CV in Opportunities/Murphy AI - Product Manager/.</t>
+          <t>Generalist PM. Archetype C — AI-native product startup, explicitly domain-agnostic. CV in Opportunities/26-08-25 - Murphy AI - Product Manager/.</t>
         </is>
       </c>
     </row>
@@ -3022,7 +3022,7 @@
       </c>
       <c r="L42" s="5" t="inlineStr">
         <is>
-          <t>Generalist PM / Archetype A-C overlap. Barcelona, 3 days onsite (relocation assistance available). The only real stretch here is "Staff" — above Senior at most companies (the band the pipeline auto-excludes as Director/Principal), but scope in the JD reads as squad-leading IC, and per the standing per-req rule ambiguous titles get called individually. Corrected framing (2026-09-07): the AI ask in this JD is not a high technical bar — it literally asks whether you work with tools like Cursor, Bolt, Claude Code, Figma, Git and prototype with them. Joaco does exactly that daily and has shipped real self-built sites (El Dugout, eldugout.vercel.app) — this is a match on evidence, not a stretch.</t>
+          <t>Generalist PM / Archetype A-C overlap. Barcelona, 3 days onsite (relocation assistance available). The only real stretch here is "Staff" — above Senior at most companies (the band the pipeline auto-excludes as Director/Principal), but scope in the JD reads as squad-leading IC, and per the standing per-req rule ambiguous titles get called individually. Corrected framing (2026-09-07): the AI ask in this JD is not a high technical bar — it literally asks whether you work with tools like Cursor, Bolt, Claude Code, Figma, Git and prototype with them. Joaco does exactly that daily and has shipped real self-built sites (The Playmaker, theplaymaker.app) — this is a match on evidence, not a stretch.</t>
         </is>
       </c>
     </row>
@@ -3193,7 +3193,7 @@
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Refresh spreadsheet — Docplanner CV built
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job Candidates.xlsx
+++ b/Job Candidates.xlsx
@@ -3321,7 +3321,11 @@
           <t>Investable Stretch (quick read, not full decode)</t>
         </is>
       </c>
-      <c r="G46" s="5" t="inlineStr"/>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>❌ Translating business logic into ranking/scoring systems (REQUIRED — never built one; the Ironhack Song Recommender is not the same thing). ❌ Two-sided marketplace dynamics (REQUIRED — Despegar was buyer-side only). ❌ Subscription metrics as owned numbers: churn, ARPU, LTV (REQUIRED — not evidenced anywhere). ❌ Pricing/monetization/ads products (bonus). ❌ Healthcare (bonus). ✅ SQL + A/B + funnel analysis. ✅ Activation — the real bridge to "zero-booking doctors".</t>
+        </is>
+      </c>
       <c r="H46" s="4" t="inlineStr">
         <is>
           <t>yes</t>
@@ -3334,7 +3338,7 @@
       </c>
       <c r="J46" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K46" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Refresh spreadsheet — Powens CV built
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job Candidates.xlsx
+++ b/Job Candidates.xlsx
@@ -3124,7 +3124,11 @@
           <t>Investable Stretch (quick read, not full decode)</t>
         </is>
       </c>
-      <c r="G43" s="5" t="inlineStr"/>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>❌ 2+ years managing product professionals (REQUIRED — he has 1 year with an APM, and the role directly manages 1-2 Product Owners reporting to the CPTO. Biggest gap). ❌ Proptech vertical — but the company is Open Finance, so the fintech-SaaS half of that requirement is met. ❌ French (nice-to-have). ⚠️ 7 years stated minimum — the CV says "6+" but his own dates total 8y5m. Met in reality, not on the page. Decide the number before sending. ✅ Native Spanish — a stated hard requirement and a real differentiator. ✅ Fintech SaaS, product-area ownership, discovery.</t>
+        </is>
+      </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
           <t>yes</t>
@@ -3137,7 +3141,7 @@
       </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K43" s="4" t="inlineStr">
@@ -3323,7 +3327,7 @@
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>❌ Translating business logic into ranking/scoring systems (REQUIRED — never built one; the Ironhack Song Recommender is not the same thing). ❌ Two-sided marketplace dynamics (REQUIRED — Despegar was buyer-side only). ❌ Subscription metrics as owned numbers: churn, ARPU, LTV (REQUIRED — not evidenced anywhere). ❌ Pricing/monetization/ads products (bonus). ❌ Healthcare (bonus). ✅ SQL + A/B + funnel analysis. ✅ Activation — the real bridge to "zero-booking doctors".</t>
+          <t>❌ Translating business logic into ranking/scoring systems (REQUIRED — never built one in production; the Ironhack Song Recommender and Airbnb Pricing Model are bootcamp exercises, not the same thing). ❌ Two-sided marketplace dynamics (REQUIRED — confirmed with Joaco 2026-09-07: one side only). ❌ Pricing/monetization/ads products (bonus). ❌ Healthcare (bonus). ✅ Subscription metrics — churn (Directv, Kantox), ARPU and LTV (Despegar, IOL). Confirmed by Joaco 2026-09-07; was missing from the CV, not from his experience. ✅ SQL + A/B + funnel analysis. ✅ Activation — the real bridge to "zero-booking doctors".</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Refresh spreadsheet — Perk CV built, queue empty
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job Candidates.xlsx
+++ b/Job Candidates.xlsx
@@ -3061,7 +3061,11 @@
           <t>Investable Stretch (quick read, not full decode) — stretch is the title band, not the skills</t>
         </is>
       </c>
-      <c r="G42" s="5" t="inlineStr"/>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>❌ Expense lifecycle from spend inception through ERP posting (REQUIRED — he has payments and checkout, not expense management, invoice processing or ERP reconciliation. The real domain gap). ❌ Leading multiple squads in parallel — he has led one squad and one Product Owner. ❌ Cursor (named in the JD; he uses Claude Code and Bolt). ⚠️ Staff title band — but LinkedIn tags the posting itself "Mid-Senior". ✅ Hands-on AI via side projects — met literally: the JD names Bolt and Claude Code, both on his CV, and The Playmaker is the shipped side project it describes. ✅ Travel + payments in one profile, which is the role's whole premise.</t>
+        </is>
+      </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
           <t>yes — Joaco's call 2026-09-07: apply anyway</t>
@@ -3074,7 +3078,7 @@
       </c>
       <c r="J42" s="4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K42" s="4" t="inlineStr">

</xml_diff>